<commit_message>
Reduced grayscale image capability
</commit_message>
<xml_diff>
--- a/inputs/radar.xlsx
+++ b/inputs/radar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\friedele\Repos\DRFM\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E5EE66-DB86-4634-9965-74148434E915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3394650B-0273-4214-B694-E040D38C6B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29940" yWindow="2040" windowWidth="15165" windowHeight="9750" xr2:uid="{E49E1DF9-4937-4C6D-9A78-CA6266DF6DC5}"/>
+    <workbookView xWindow="32700" yWindow="2310" windowWidth="17580" windowHeight="8955" xr2:uid="{E49E1DF9-4937-4C6D-9A78-CA6266DF6DC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Pri</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t>pwEnum</t>
+  </si>
+  <si>
+    <t>noiseFigure</t>
   </si>
 </sst>
 </file>
@@ -440,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21C0482-AC5F-49E4-B7B5-F9FEEC654263}">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="8.7109375" customWidth="1"/>
@@ -452,9 +455,10 @@
     <col min="11" max="11" width="10.42578125" customWidth="1"/>
     <col min="12" max="12" width="7.85546875" customWidth="1"/>
     <col min="13" max="13" width="7.140625" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -494,8 +498,11 @@
       <c r="M1" t="s">
         <v>5</v>
       </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -507,7 +514,7 @@
         <v>0.25</v>
       </c>
       <c r="D2" s="3">
-        <v>9000000000</v>
+        <v>9500000000</v>
       </c>
       <c r="E2" s="4">
         <f>1/F2</f>
@@ -532,13 +539,16 @@
         <v>450000</v>
       </c>
       <c r="L2" s="2">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="M2" s="2">
-        <v>120</v>
+        <v>100</v>
+      </c>
+      <c r="N2" s="5">
+        <v>1E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -580,8 +590,11 @@
       <c r="M3" s="2">
         <v>100</v>
       </c>
+      <c r="N3" s="5">
+        <v>1E-3</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -623,8 +636,11 @@
       <c r="M4" s="2">
         <v>100</v>
       </c>
+      <c r="N4" s="5">
+        <v>1E-3</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -666,8 +682,11 @@
       <c r="M5" s="2">
         <v>90</v>
       </c>
+      <c r="N5" s="5">
+        <v>1E-3</v>
+      </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -709,8 +728,11 @@
       <c r="M6" s="2">
         <v>70</v>
       </c>
+      <c r="N6" s="5">
+        <v>1E-3</v>
+      </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -752,8 +774,11 @@
       <c r="M7" s="2">
         <v>60</v>
       </c>
+      <c r="N7" s="5">
+        <v>1E-3</v>
+      </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="I13" s="1"/>
     </row>
   </sheetData>

</xml_diff>